<commit_message>
feat(curriculum): roll concept mappings up to competency and goal
load_frame() denormalises ancestry only downward, so a learning outcome
carries its competency and goal but a competency carries only its goal and a
goal carries neither. _ancestry() makes both columns answerable for every row
by treating a row as its own competency when it IS one, and its own goal when
it IS one.

A concept matched to a competency also serves the outcomes stated beneath it,
so _inherited_from_competencies() writes those with match_source='inherited'
and a score well below anything the model or the lexical matcher produces --
'inherited' is the value this column's COMMENT has documented since the table
was created.

Backs 31,743 rows in lms_concept_outcome across standards 39-43; verify.py
returns 0 on all three checks for each.

Migration numbered 009: master already holds an 008.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/queue/class7_cbse_queue.xlsx
+++ b/backend/queue/class7_cbse_queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'queue'!$A$1:$S$1</definedName>
@@ -600,14 +600,32 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>342</v>
+      </c>
+      <c r="M2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N2" t="n">
+        <v>10504</v>
+      </c>
+      <c r="O2" t="n">
+        <v>12</v>
+      </c>
+      <c r="P2" t="n">
+        <v>199.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:21:15</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -654,19 +672,33 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>343</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>27497</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>478.7</v>
+      </c>
       <c r="Q3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:29:15</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -713,14 +745,32 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>344</v>
+      </c>
+      <c r="M4" t="n">
+        <v>18</v>
+      </c>
+      <c r="N4" t="n">
+        <v>30174</v>
+      </c>
+      <c r="O4" t="n">
+        <v>44</v>
+      </c>
+      <c r="P4" t="n">
+        <v>396.4</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:35:54</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -767,19 +817,33 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
-      <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>345</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>27387</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>380.8</v>
+      </c>
       <c r="Q5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:42:16</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -826,14 +890,32 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>346</v>
+      </c>
+      <c r="M6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N6" t="n">
+        <v>25529</v>
+      </c>
+      <c r="O6" t="n">
+        <v>24</v>
+      </c>
+      <c r="P6" t="n">
+        <v>404</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:49:01</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -880,19 +962,33 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>347</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>28069</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>497.7</v>
+      </c>
       <c r="Q7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:57:20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -939,14 +1035,32 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>349</v>
+      </c>
+      <c r="M8" t="n">
+        <v>16</v>
+      </c>
+      <c r="N8" t="n">
+        <v>30986</v>
+      </c>
+      <c r="O8" t="n">
+        <v>37</v>
+      </c>
+      <c r="P8" t="n">
+        <v>437.4</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2026-09-19T11:04:38</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -993,19 +1107,33 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
-      <c r="O9" s="2" t="n"/>
-      <c r="P9" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>30068</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>576</v>
+      </c>
       <c r="Q9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T11:14:16</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1052,14 +1180,32 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>352</v>
+      </c>
+      <c r="M10" t="n">
+        <v>16</v>
+      </c>
+      <c r="N10" t="n">
+        <v>32148</v>
+      </c>
+      <c r="O10" t="n">
+        <v>30</v>
+      </c>
+      <c r="P10" t="n">
+        <v>333.8</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2026-09-19T11:19:54</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1106,19 +1252,33 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="n"/>
-      <c r="P11" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>353</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>29449</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>594.1</v>
+      </c>
       <c r="Q11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T11:29:50</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1165,14 +1325,32 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>360</v>
+      </c>
+      <c r="M12" t="n">
+        <v>16</v>
+      </c>
+      <c r="N12" t="n">
+        <v>29843</v>
+      </c>
+      <c r="O12" t="n">
+        <v>40</v>
+      </c>
+      <c r="P12" t="n">
+        <v>592.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>2026-09-19T13:54:00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1219,19 +1397,33 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>35268</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>302.6</v>
+      </c>
       <c r="Q13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T13:59:04</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1278,14 +1470,32 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>362</v>
+      </c>
+      <c r="M14" t="n">
+        <v>42</v>
+      </c>
+      <c r="N14" t="n">
+        <v>60409</v>
+      </c>
+      <c r="O14" t="n">
+        <v>46</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1487.6</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>2026-09-19T14:23:54</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1332,19 +1542,33 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="n"/>
-      <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>363</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>67816</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>1224.5</v>
+      </c>
       <c r="Q15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T14:44:21</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1391,14 +1615,32 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>364</v>
+      </c>
+      <c r="M16" t="n">
+        <v>48</v>
+      </c>
+      <c r="N16" t="n">
+        <v>69744</v>
+      </c>
+      <c r="O16" t="n">
+        <v>54</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1762.1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:13:46</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1445,19 +1687,33 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>365</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>61692</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>933.4</v>
+      </c>
       <c r="Q17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T15:29:21</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1504,14 +1760,32 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>366</v>
+      </c>
+      <c r="M18" t="n">
+        <v>47</v>
+      </c>
+      <c r="N18" t="n">
+        <v>64705</v>
+      </c>
+      <c r="O18" t="n">
+        <v>46</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1898.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:01:01</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1558,14 +1832,32 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>376</v>
+      </c>
+      <c r="M19" t="n">
+        <v>13</v>
+      </c>
+      <c r="N19" t="n">
+        <v>11959</v>
+      </c>
+      <c r="O19" t="n">
+        <v>23</v>
+      </c>
+      <c r="P19" t="n">
+        <v>512.8</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:09:35</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1612,19 +1904,33 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>377</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>17557</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>357.8</v>
+      </c>
       <c r="Q20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:15:34</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1671,14 +1977,32 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>379</v>
+      </c>
+      <c r="M21" t="n">
+        <v>12</v>
+      </c>
+      <c r="N21" t="n">
+        <v>11850</v>
+      </c>
+      <c r="O21" t="n">
+        <v>23</v>
+      </c>
+      <c r="P21" t="n">
+        <v>472.1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:23:28</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1725,19 +2049,33 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="n"/>
-      <c r="N22" s="2" t="n"/>
-      <c r="O22" s="2" t="n"/>
-      <c r="P22" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>18624</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>435.5</v>
+      </c>
       <c r="Q22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:30:45</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1784,14 +2122,32 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>381</v>
+      </c>
+      <c r="M23" t="n">
+        <v>16</v>
+      </c>
+      <c r="N23" t="n">
+        <v>17090</v>
+      </c>
+      <c r="O23" t="n">
+        <v>20</v>
+      </c>
+      <c r="P23" t="n">
+        <v>536.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:39:43</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1838,19 +2194,33 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="n"/>
-      <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>382</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>9831</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>1301.7</v>
+      </c>
       <c r="Q24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T17:01:26</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1897,14 +2267,32 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>384</v>
+      </c>
+      <c r="M25" t="n">
+        <v>13</v>
+      </c>
+      <c r="N25" t="n">
+        <v>12699</v>
+      </c>
+      <c r="O25" t="n">
+        <v>22</v>
+      </c>
+      <c r="P25" t="n">
+        <v>285.2</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>2026-09-19T17:06:13</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1951,19 +2339,33 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="n"/>
-      <c r="P26" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>385</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>23974</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>368.9</v>
+      </c>
       <c r="Q26" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T17:12:23</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2010,14 +2412,32 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>386</v>
+      </c>
+      <c r="M27" t="n">
+        <v>12</v>
+      </c>
+      <c r="N27" t="n">
+        <v>11732</v>
+      </c>
+      <c r="O27" t="n">
+        <v>18</v>
+      </c>
+      <c r="P27" t="n">
+        <v>226.3</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>2026-09-19T17:16:11</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2064,19 +2484,33 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="n"/>
-      <c r="M28" s="2" t="n"/>
-      <c r="N28" s="2" t="n"/>
-      <c r="O28" s="2" t="n"/>
-      <c r="P28" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>514</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>24237</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>2326.8</v>
+      </c>
       <c r="Q28" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T10:43:07</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2123,14 +2557,32 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>388</v>
+      </c>
+      <c r="M29" t="n">
+        <v>38</v>
+      </c>
+      <c r="N29" t="n">
+        <v>56560</v>
+      </c>
+      <c r="O29" t="n">
+        <v>42</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1363.2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>2026-09-19T17:40:29</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2177,19 +2629,33 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="n"/>
-      <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="n"/>
-      <c r="P30" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>390</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>62670</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>808.2</v>
+      </c>
       <c r="Q30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" s="2" t="inlineStr"/>
-      <c r="S30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T17:54:00</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2236,14 +2702,32 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>391</v>
+      </c>
+      <c r="M31" t="n">
+        <v>55</v>
+      </c>
+      <c r="N31" t="n">
+        <v>66953</v>
+      </c>
+      <c r="O31" t="n">
+        <v>100</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1887.8</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:25:29</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2290,19 +2774,33 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>392</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>67914</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>1975.8</v>
+      </c>
       <c r="Q32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R32" s="2" t="inlineStr"/>
-      <c r="S32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T18:58:28</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2349,14 +2847,32 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>394</v>
+      </c>
+      <c r="M33" t="n">
+        <v>34</v>
+      </c>
+      <c r="N33" t="n">
+        <v>41578</v>
+      </c>
+      <c r="O33" t="n">
+        <v>72</v>
+      </c>
+      <c r="P33" t="n">
+        <v>642.9</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>2026-09-19T19:09:11</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2403,19 +2919,33 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>404</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>51364</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>1279.4</v>
+      </c>
       <c r="Q34" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T19:30:32</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2462,14 +2992,32 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>405</v>
+      </c>
+      <c r="M35" t="n">
+        <v>34</v>
+      </c>
+      <c r="N35" t="n">
+        <v>51038</v>
+      </c>
+      <c r="O35" t="n">
+        <v>63</v>
+      </c>
+      <c r="P35" t="n">
+        <v>588.8</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>2026-09-19T19:40:22</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2516,19 +3064,33 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>406</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>52672</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>1062</v>
+      </c>
       <c r="Q36" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R36" s="2" t="inlineStr"/>
-      <c r="S36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T19:58:04</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2575,14 +3137,32 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>412</v>
+      </c>
+      <c r="M37" t="n">
+        <v>23</v>
+      </c>
+      <c r="N37" t="n">
+        <v>31510</v>
+      </c>
+      <c r="O37" t="n">
+        <v>59</v>
+      </c>
+      <c r="P37" t="n">
+        <v>375.2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>2026-09-19T20:04:20</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2629,19 +3209,33 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-      <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="n"/>
-      <c r="P38" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>39772</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>1258.1</v>
+      </c>
       <c r="Q38" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R38" s="2" t="inlineStr"/>
-      <c r="S38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T20:25:20</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2688,14 +3282,32 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>414</v>
+      </c>
+      <c r="M39" t="n">
+        <v>20</v>
+      </c>
+      <c r="N39" t="n">
+        <v>37059</v>
+      </c>
+      <c r="O39" t="n">
+        <v>38</v>
+      </c>
+      <c r="P39" t="n">
+        <v>511.8</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>2026-09-19T20:33:52</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2742,19 +3354,33 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="n"/>
-      <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="n"/>
-      <c r="P40" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>415</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>44063</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>1752</v>
+      </c>
       <c r="Q40" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R40" s="2" t="inlineStr"/>
-      <c r="S40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T21:03:05</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2801,14 +3427,32 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>416</v>
+      </c>
+      <c r="M41" t="n">
+        <v>39</v>
+      </c>
+      <c r="N41" t="n">
+        <v>59982</v>
+      </c>
+      <c r="O41" t="n">
+        <v>78</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2241.5</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>2026-09-19T21:40:27</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2855,19 +3499,33 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="n"/>
-      <c r="N42" s="2" t="n"/>
-      <c r="O42" s="2" t="n"/>
-      <c r="P42" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>417</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>41128</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>526.4</v>
+      </c>
       <c r="Q42" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R42" s="2" t="inlineStr"/>
-      <c r="S42" s="2" t="inlineStr"/>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T21:49:15</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2914,14 +3572,32 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>418</v>
+      </c>
+      <c r="M43" t="n">
+        <v>31</v>
+      </c>
+      <c r="N43" t="n">
+        <v>50160</v>
+      </c>
+      <c r="O43" t="n">
+        <v>51</v>
+      </c>
+      <c r="P43" t="n">
+        <v>3652.2</v>
       </c>
       <c r="Q43" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:50:08</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2968,14 +3644,32 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>419</v>
+      </c>
+      <c r="M44" t="n">
+        <v>26</v>
+      </c>
+      <c r="N44" t="n">
+        <v>29858</v>
+      </c>
+      <c r="O44" t="n">
+        <v>45</v>
+      </c>
+      <c r="P44" t="n">
+        <v>455.6</v>
       </c>
       <c r="Q44" t="n">
-        <v>0</v>
-      </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>2026-09-19T22:57:44</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3022,19 +3716,33 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="n"/>
-      <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n"/>
-      <c r="P45" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="M45" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>23912</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>914.6</v>
+      </c>
       <c r="Q45" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R45" s="2" t="inlineStr"/>
-      <c r="S45" s="2" t="inlineStr"/>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:12:59</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3081,14 +3789,32 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>421</v>
+      </c>
+      <c r="M46" t="n">
+        <v>22</v>
+      </c>
+      <c r="N46" t="n">
+        <v>30604</v>
+      </c>
+      <c r="O46" t="n">
+        <v>20</v>
+      </c>
+      <c r="P46" t="n">
+        <v>454.4</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
-      </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:20:34</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3135,19 +3861,33 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="n"/>
-      <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="n"/>
-      <c r="P47" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>422</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N47" s="2" t="n">
+        <v>18667</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>329.2</v>
+      </c>
       <c r="Q47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R47" s="2" t="inlineStr"/>
-      <c r="S47" s="2" t="inlineStr"/>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:26:04</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3194,14 +3934,32 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
+        <v>423</v>
+      </c>
+      <c r="M48" t="n">
+        <v>33</v>
+      </c>
+      <c r="N48" t="n">
+        <v>39849</v>
+      </c>
+      <c r="O48" t="n">
+        <v>44</v>
+      </c>
+      <c r="P48" t="n">
+        <v>483.8</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:34:08</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3248,19 +4006,33 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="n"/>
-      <c r="N49" s="2" t="n"/>
-      <c r="O49" s="2" t="n"/>
-      <c r="P49" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>424</v>
+      </c>
+      <c r="M49" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="N49" s="2" t="n">
+        <v>31250</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>492.5</v>
+      </c>
       <c r="Q49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R49" s="2" t="inlineStr"/>
-      <c r="S49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:42:21</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3307,14 +4079,32 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
+        <v>425</v>
+      </c>
+      <c r="M50" t="n">
+        <v>22</v>
+      </c>
+      <c r="N50" t="n">
+        <v>28130</v>
+      </c>
+      <c r="O50" t="n">
+        <v>21</v>
+      </c>
+      <c r="P50" t="n">
+        <v>453.6</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
-      </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:49:55</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3361,19 +4151,33 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="n"/>
-      <c r="M51" s="2" t="n"/>
-      <c r="N51" s="2" t="n"/>
-      <c r="O51" s="2" t="n"/>
-      <c r="P51" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>26117</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>353.2</v>
+      </c>
       <c r="Q51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R51" s="2" t="inlineStr"/>
-      <c r="S51" s="2" t="inlineStr"/>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:55:49</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3420,14 +4224,32 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
+        <v>427</v>
+      </c>
+      <c r="M52" t="n">
+        <v>24</v>
+      </c>
+      <c r="N52" t="n">
+        <v>38138</v>
+      </c>
+      <c r="O52" t="n">
+        <v>25</v>
+      </c>
+      <c r="P52" t="n">
+        <v>974.1</v>
       </c>
       <c r="Q52" t="n">
-        <v>0</v>
-      </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>2026-09-20T00:12:04</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3474,19 +4296,33 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="n"/>
-      <c r="M53" s="2" t="n"/>
-      <c r="N53" s="2" t="n"/>
-      <c r="O53" s="2" t="n"/>
-      <c r="P53" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="n">
+        <v>428</v>
+      </c>
+      <c r="M53" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>26071</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="P53" s="2" t="n">
+        <v>649.2</v>
+      </c>
       <c r="Q53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R53" s="2" t="inlineStr"/>
-      <c r="S53" s="2" t="inlineStr"/>
+      <c r="S53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T00:22:54</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3533,14 +4369,32 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>429</v>
+      </c>
+      <c r="M54" t="n">
+        <v>18</v>
+      </c>
+      <c r="N54" t="n">
+        <v>22800</v>
+      </c>
+      <c r="O54" t="n">
+        <v>26</v>
+      </c>
+      <c r="P54" t="n">
+        <v>326</v>
       </c>
       <c r="Q54" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>2026-09-20T00:28:21</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3587,19 +4441,33 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="n"/>
-      <c r="M55" s="2" t="n"/>
-      <c r="N55" s="2" t="n"/>
-      <c r="O55" s="2" t="n"/>
-      <c r="P55" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>430</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>34279</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>655.5</v>
+      </c>
       <c r="Q55" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R55" s="2" t="inlineStr"/>
-      <c r="S55" s="2" t="inlineStr"/>
+      <c r="S55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T00:39:17</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3646,14 +4514,32 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>431</v>
+      </c>
+      <c r="M56" t="n">
+        <v>28</v>
+      </c>
+      <c r="N56" t="n">
+        <v>37566</v>
+      </c>
+      <c r="O56" t="n">
+        <v>23</v>
+      </c>
+      <c r="P56" t="n">
+        <v>548.7</v>
       </c>
       <c r="Q56" t="n">
-        <v>0</v>
-      </c>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>2026-09-20T00:48:27</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3700,19 +4586,33 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="n"/>
-      <c r="M57" s="2" t="n"/>
-      <c r="N57" s="2" t="n"/>
-      <c r="O57" s="2" t="n"/>
-      <c r="P57" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="M57" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="N57" s="2" t="n">
+        <v>42697</v>
+      </c>
+      <c r="O57" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="P57" s="2" t="n">
+        <v>489.6</v>
+      </c>
       <c r="Q57" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R57" s="2" t="inlineStr"/>
-      <c r="S57" s="2" t="inlineStr"/>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T00:56:37</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3759,14 +4659,32 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>433</v>
+      </c>
+      <c r="M58" t="n">
+        <v>36</v>
+      </c>
+      <c r="N58" t="n">
+        <v>55903</v>
+      </c>
+      <c r="O58" t="n">
+        <v>28</v>
+      </c>
+      <c r="P58" t="n">
+        <v>628.6</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:07:06</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3813,19 +4731,33 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="n"/>
-      <c r="M59" s="2" t="n"/>
-      <c r="N59" s="2" t="n"/>
-      <c r="O59" s="2" t="n"/>
-      <c r="P59" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>434</v>
+      </c>
+      <c r="M59" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>41916</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>478.3</v>
+      </c>
       <c r="Q59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R59" s="2" t="inlineStr"/>
-      <c r="S59" s="2" t="inlineStr"/>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:15:05</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3872,14 +4804,32 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
+        <v>435</v>
+      </c>
+      <c r="M60" t="n">
+        <v>18</v>
+      </c>
+      <c r="N60" t="n">
+        <v>25753</v>
+      </c>
+      <c r="O60" t="n">
+        <v>18</v>
+      </c>
+      <c r="P60" t="n">
+        <v>330.9</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
-      </c>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:20:37</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3926,19 +4876,33 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="n"/>
-      <c r="M61" s="2" t="n"/>
-      <c r="N61" s="2" t="n"/>
-      <c r="O61" s="2" t="n"/>
-      <c r="P61" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="n">
+        <v>436</v>
+      </c>
+      <c r="M61" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="N61" s="2" t="n">
+        <v>36829</v>
+      </c>
+      <c r="O61" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="P61" s="2" t="n">
+        <v>604.6</v>
+      </c>
       <c r="Q61" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R61" s="2" t="inlineStr"/>
-      <c r="S61" s="2" t="inlineStr"/>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:30:43</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3985,14 +4949,32 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
+        <v>437</v>
+      </c>
+      <c r="M62" t="n">
+        <v>24</v>
+      </c>
+      <c r="N62" t="n">
+        <v>27901</v>
+      </c>
+      <c r="O62" t="n">
+        <v>38</v>
+      </c>
+      <c r="P62" t="n">
+        <v>365.5</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
-      </c>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:36:49</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4039,19 +5021,33 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="n"/>
-      <c r="M63" s="2" t="n"/>
-      <c r="N63" s="2" t="n"/>
-      <c r="O63" s="2" t="n"/>
-      <c r="P63" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="n">
+        <v>438</v>
+      </c>
+      <c r="M63" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>27564</v>
+      </c>
+      <c r="O63" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="P63" s="2" t="n">
+        <v>357.2</v>
+      </c>
       <c r="Q63" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R63" s="2" t="inlineStr"/>
-      <c r="S63" s="2" t="inlineStr"/>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:42:47</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>

</xml_diff>